<commit_message>
Add AI budget guidance and confirm Jeju dates
</commit_message>
<xml_diff>
--- a/outputs/019fa660-42f1-74a1-ab98-31c99abb6300/韩国济州岛旅行共创.xlsx
+++ b/outputs/019fa660-42f1-74a1-ab98-31c99abb6300/韩国济州岛旅行共创.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1600" uniqueCount="681">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1601" uniqueCount="681">
   <si>
     <t>韩国济州岛旅行 · 最终方案首页</t>
   </si>
@@ -36,7 +36,7 @@
     <t>网站只读取这一页作为最终攻略；后面的工作表都是候选资料和处理记录。</t>
   </si>
   <si>
-    <t>黄色单元格可直接修改；保存 Excel 后约 4 秒同步网站。当前已确定 14/18 项，待补充 4 项。</t>
+    <t>黄色单元格可直接修改；保存 Excel 后约 4 秒同步网站。当前已确定 15/18 项，待补充 3 项。</t>
   </si>
   <si>
     <t>一、基础信息  ·  网站顶部与旅行概览</t>
@@ -66,63 +66,63 @@
     <t>出行日期</t>
   </si>
   <si>
-    <t>待团队确认</t>
+    <t>2026年8月21日–23日（周五–周日）</t>
+  </si>
+  <si>
+    <t>确定日期后直接在黄色单元格修改</t>
+  </si>
+  <si>
+    <t>行程结构</t>
+  </si>
+  <si>
+    <t>3 天 2 晚 · 国际航班直达济州</t>
+  </si>
+  <si>
+    <t>例如：3 天 2 晚 · 国际航班直达济州</t>
+  </si>
+  <si>
+    <t>同行人数</t>
+  </si>
+  <si>
+    <t>用于住宿、餐饮和活动人数判断</t>
+  </si>
+  <si>
+    <t>住宿晚数</t>
+  </si>
+  <si>
+    <t>当前按 3 天 2 晚设计</t>
+  </si>
+  <si>
+    <t>人均预算</t>
+  </si>
+  <si>
+    <t>¥1,000–1,500 / 人（不含往返济州机票）</t>
+  </si>
+  <si>
+    <t>可填写数字或预算区间</t>
+  </si>
+  <si>
+    <t>方案说明</t>
+  </si>
+  <si>
+    <t>六人按真实消费重算：正餐约 ¥100/人，穿插民宿做饭与一起吃宵夜；岛内公交优先、必要时短途拼车，不默认全程打车或包车；贵景点可换成免费海岸、市场和步道。</t>
+  </si>
+  <si>
+    <t>网站首页的行程摘要</t>
+  </si>
+  <si>
+    <t>二、住宿确认  ·  民宿未确定前保持橙色“待补充”</t>
+  </si>
+  <si>
+    <t>民宿名称</t>
+  </si>
+  <si>
+    <t>待选择｜济州市区六人酒店或公寓</t>
   </si>
   <si>
     <t>待补充</t>
   </si>
   <si>
-    <t>确定日期后直接在黄色单元格修改</t>
-  </si>
-  <si>
-    <t>行程结构</t>
-  </si>
-  <si>
-    <t>3 天 2 晚 · 国际航班直达济州</t>
-  </si>
-  <si>
-    <t>例如：3 天 2 晚 · 国际航班直达济州</t>
-  </si>
-  <si>
-    <t>同行人数</t>
-  </si>
-  <si>
-    <t>用于住宿、餐饮和活动人数判断</t>
-  </si>
-  <si>
-    <t>住宿晚数</t>
-  </si>
-  <si>
-    <t>当前按 3 天 2 晚设计</t>
-  </si>
-  <si>
-    <t>人均预算</t>
-  </si>
-  <si>
-    <t>¥1,000–1,500 / 人（不含往返济州机票）</t>
-  </si>
-  <si>
-    <t>可填写数字或预算区间</t>
-  </si>
-  <si>
-    <t>方案说明</t>
-  </si>
-  <si>
-    <t>六人按真实消费重算：正餐约 ¥100/人，穿插民宿做饭与一起吃宵夜；岛内公交优先、必要时短途拼车，不默认全程打车或包车；贵景点可换成免费海岸、市场和步道。</t>
-  </si>
-  <si>
-    <t>网站首页的行程摘要</t>
-  </si>
-  <si>
-    <t>二、住宿确认  ·  民宿未确定前保持橙色“待补充”</t>
-  </si>
-  <si>
-    <t>民宿名称</t>
-  </si>
-  <si>
-    <t>待选择｜济州市区六人酒店或公寓</t>
-  </si>
-  <si>
     <t>确定住宿后填写真实名称</t>
   </si>
   <si>
@@ -579,7 +579,7 @@
     <t>reserve-dates-flight</t>
   </si>
   <si>
-    <t>确定日期与国际直达济州往返航班</t>
+    <t>预订国际直达济州往返航班</t>
   </si>
   <si>
     <t>机票</t>
@@ -591,7 +591,7 @@
     <t>待认领</t>
   </si>
   <si>
-    <t>优先完成</t>
+    <t>尽快确认</t>
   </si>
   <si>
     <t>不要购买经首尔转韩国国内线的方案；六人的去回航班与行李额需统一</t>
@@ -624,9 +624,6 @@
     <t>待补充真实链接</t>
   </si>
   <si>
-    <t>日期确认后立即</t>
-  </si>
-  <si>
     <t>比较房型、床型、含税总价、位置、取消政策和延迟入住限制</t>
   </si>
   <si>
@@ -921,6 +918,9 @@
     <t>请团队优先投递 3–5 个真实住宿链接</t>
   </si>
   <si>
+    <t>priceLabel</t>
+  </si>
+  <si>
     <t>文字</t>
   </si>
   <si>
@@ -2067,7 +2067,7 @@
     <t>当前重点</t>
   </si>
   <si>
-    <t>确定日期与直达航班、住宿、包车和具体餐厅</t>
+    <t>确定日期与直达航班、住宿、公交班次和具体餐厅</t>
   </si>
   <si>
     <t>可投递链接，也可直接写文字诉求</t>
@@ -2853,11 +2853,11 @@
         <v>12</v>
       </c>
       <c r="C8" s="6"/>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" s="8" t="s">
         <v>13</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>14</v>
       </c>
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
@@ -2869,17 +2869,17 @@
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>15</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>16</v>
       </c>
       <c r="C9" s="6"/>
       <c r="D9" s="7" t="s">
         <v>6</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
@@ -2891,7 +2891,7 @@
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B10" s="6">
         <v>6</v>
@@ -2901,7 +2901,7 @@
         <v>6</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F10" s="8"/>
       <c r="G10" s="8"/>
@@ -2913,7 +2913,7 @@
     </row>
     <row r="11" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B11" s="6">
         <v>2</v>
@@ -2923,7 +2923,7 @@
         <v>6</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F11" s="8"/>
       <c r="G11" s="8"/>
@@ -2935,17 +2935,17 @@
     </row>
     <row r="12" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="6" t="s">
         <v>22</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>23</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="7" t="s">
         <v>6</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F12" s="8"/>
       <c r="G12" s="8"/>
@@ -2957,17 +2957,17 @@
     </row>
     <row r="13" ht="46" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>25</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>26</v>
       </c>
       <c r="C13" s="6"/>
       <c r="D13" s="7" t="s">
         <v>6</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
@@ -2979,7 +2979,7 @@
     </row>
     <row r="15" ht="30" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -2995,14 +2995,14 @@
     </row>
     <row r="16" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" s="6" t="s">
         <v>29</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>30</v>
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="9" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="E16" s="8" t="s">
         <v>31</v>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="C17" s="6"/>
       <c r="D17" s="9" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="E17" s="8" t="s">
         <v>34</v>
@@ -3198,7 +3198,7 @@
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
       <c r="D25" s="9" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="E25" s="8" t="s">
         <v>57</v>
@@ -3859,50 +3859,50 @@
         <v>186</v>
       </c>
       <c r="G47" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="H47" s="11" t="s">
         <v>198</v>
-      </c>
-      <c r="H47" s="11" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="48" ht="38" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="B48" s="14" t="s">
         <v>200</v>
-      </c>
-      <c r="B48" s="14" t="s">
-        <v>201</v>
       </c>
       <c r="C48" s="14" t="s">
         <v>66</v>
       </c>
       <c r="D48" s="14" t="s">
+        <v>201</v>
+      </c>
+      <c r="E48" s="14" t="s">
         <v>202</v>
-      </c>
-      <c r="E48" s="14" t="s">
-        <v>203</v>
       </c>
       <c r="F48" s="14" t="s">
         <v>186</v>
       </c>
       <c r="G48" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="H48" s="14" t="s">
         <v>204</v>
-      </c>
-      <c r="H48" s="14" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="49" ht="38" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
+        <v>205</v>
+      </c>
+      <c r="B49" s="11" t="s">
         <v>206</v>
       </c>
-      <c r="B49" s="11" t="s">
+      <c r="C49" s="11" t="s">
         <v>207</v>
       </c>
-      <c r="C49" s="11" t="s">
+      <c r="D49" s="11" t="s">
         <v>208</v>
-      </c>
-      <c r="D49" s="11" t="s">
-        <v>209</v>
       </c>
       <c r="E49" s="11" t="s">
         <v>197</v>
@@ -3911,24 +3911,24 @@
         <v>186</v>
       </c>
       <c r="G49" s="11" t="s">
+        <v>209</v>
+      </c>
+      <c r="H49" s="11" t="s">
         <v>210</v>
-      </c>
-      <c r="H49" s="11" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="50" ht="38" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
+        <v>211</v>
+      </c>
+      <c r="B50" s="14" t="s">
         <v>212</v>
       </c>
-      <c r="B50" s="14" t="s">
+      <c r="C50" s="14" t="s">
         <v>213</v>
       </c>
-      <c r="C50" s="14" t="s">
+      <c r="D50" s="14" t="s">
         <v>214</v>
-      </c>
-      <c r="D50" s="14" t="s">
-        <v>215</v>
       </c>
       <c r="E50" s="14" t="s">
         <v>79</v>
@@ -3937,10 +3937,10 @@
         <v>186</v>
       </c>
       <c r="G50" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="H50" s="14" t="s">
         <v>216</v>
-      </c>
-      <c r="H50" s="14" t="s">
-        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -4119,13 +4119,13 @@
         <v>175</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E3" s="21" t="s">
         <v>487</v>
@@ -4173,46 +4173,46 @@
         <v>509</v>
       </c>
       <c r="T3" s="22" t="s">
+        <v>230</v>
+      </c>
+      <c r="U3" s="21" t="s">
         <v>231</v>
-      </c>
-      <c r="U3" s="21" t="s">
-        <v>232</v>
       </c>
       <c r="V3" s="21" t="s">
         <v>510</v>
       </c>
       <c r="W3" s="21" t="s">
+        <v>233</v>
+      </c>
+      <c r="X3" s="21" t="s">
         <v>234</v>
       </c>
-      <c r="X3" s="21" t="s">
+      <c r="Y3" s="21" t="s">
         <v>235</v>
-      </c>
-      <c r="Y3" s="21" t="s">
-        <v>236</v>
       </c>
       <c r="Z3" s="21" t="s">
         <v>511</v>
       </c>
       <c r="AA3" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="AB3" s="21" t="s">
         <v>237</v>
       </c>
-      <c r="AB3" s="21" t="s">
+      <c r="AC3" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="AC3" s="21" t="s">
+      <c r="AD3" s="21" t="s">
         <v>239</v>
       </c>
-      <c r="AD3" s="21" t="s">
+      <c r="AE3" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="AE3" s="21" t="s">
+      <c r="AF3" s="21" t="s">
         <v>241</v>
       </c>
-      <c r="AF3" s="21" t="s">
+      <c r="AG3" s="21" t="s">
         <v>242</v>
-      </c>
-      <c r="AG3" s="21" t="s">
-        <v>243</v>
       </c>
       <c r="AH3" s="21" t="s">
         <v>512</v>
@@ -4220,26 +4220,26 @@
     </row>
     <row r="4" ht="34" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A4" s="24" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B4" s="32" t="s">
+        <v>263</v>
+      </c>
+      <c r="C4" s="32" t="s">
+        <v>262</v>
+      </c>
+      <c r="D4" s="32" t="s">
+        <v>267</v>
+      </c>
+      <c r="E4" s="32" t="s">
         <v>264</v>
-      </c>
-      <c r="C4" s="32" t="s">
-        <v>263</v>
-      </c>
-      <c r="D4" s="32" t="s">
-        <v>268</v>
-      </c>
-      <c r="E4" s="32" t="s">
-        <v>265</v>
       </c>
       <c r="F4" s="32" t="s">
         <v>122</v>
       </c>
       <c r="G4" s="35"/>
       <c r="H4" s="32" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="I4" s="32" t="s">
         <v>561</v>
@@ -4278,7 +4278,7 @@
         <v>1</v>
       </c>
       <c r="U4" s="24" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="V4" s="24" t="s">
         <v>569</v>
@@ -4294,17 +4294,17 @@
       </c>
       <c r="Z4" s="24"/>
       <c r="AA4" s="24" t="s">
+        <v>256</v>
+      </c>
+      <c r="AB4" s="24" t="s">
         <v>257</v>
       </c>
-      <c r="AB4" s="24" t="s">
-        <v>258</v>
-      </c>
       <c r="AC4" s="24" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="AD4" s="24"/>
       <c r="AE4" s="24" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="AF4" s="24"/>
       <c r="AG4" s="24" t="s">
@@ -4322,13 +4322,13 @@
         <v>323</v>
       </c>
       <c r="C5" s="32" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D5" s="32" t="s">
         <v>326</v>
       </c>
       <c r="E5" s="32" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F5" s="32" t="s">
         <v>138</v>
@@ -4390,17 +4390,17 @@
       </c>
       <c r="Z5" s="14"/>
       <c r="AA5" s="14" t="s">
+        <v>256</v>
+      </c>
+      <c r="AB5" s="14" t="s">
         <v>257</v>
-      </c>
-      <c r="AB5" s="14" t="s">
-        <v>258</v>
       </c>
       <c r="AC5" s="14" t="s">
         <v>330</v>
       </c>
       <c r="AD5" s="14"/>
       <c r="AE5" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="AF5" s="14"/>
       <c r="AG5" s="14" t="s">
@@ -4424,7 +4424,7 @@
         <v>346</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F6" s="32" t="s">
         <v>579</v>
@@ -4486,17 +4486,17 @@
       </c>
       <c r="Z6" s="24"/>
       <c r="AA6" s="24" t="s">
+        <v>256</v>
+      </c>
+      <c r="AB6" s="24" t="s">
         <v>257</v>
-      </c>
-      <c r="AB6" s="24" t="s">
-        <v>258</v>
       </c>
       <c r="AC6" s="24" t="s">
         <v>350</v>
       </c>
       <c r="AD6" s="24"/>
       <c r="AE6" s="24" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="AF6" s="24"/>
       <c r="AG6" s="24" t="s">
@@ -4514,7 +4514,7 @@
         <v>332</v>
       </c>
       <c r="C7" s="32" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D7" s="32" t="s">
         <v>336</v>
@@ -4582,17 +4582,17 @@
       </c>
       <c r="Z7" s="14"/>
       <c r="AA7" s="14" t="s">
+        <v>256</v>
+      </c>
+      <c r="AB7" s="14" t="s">
         <v>257</v>
-      </c>
-      <c r="AB7" s="14" t="s">
-        <v>258</v>
       </c>
       <c r="AC7" s="14" t="s">
         <v>340</v>
       </c>
       <c r="AD7" s="14"/>
       <c r="AE7" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="AF7" s="14"/>
       <c r="AG7" s="14" t="s">
@@ -4643,7 +4643,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -4703,10 +4703,10 @@
         <v>598</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E3" s="21" t="s">
         <v>599</v>
@@ -4721,46 +4721,46 @@
         <v>382</v>
       </c>
       <c r="I3" s="21" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J3" s="22" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="K3" s="21" t="s">
         <v>510</v>
       </c>
       <c r="L3" s="21" t="s">
+        <v>233</v>
+      </c>
+      <c r="M3" s="21" t="s">
         <v>234</v>
       </c>
-      <c r="M3" s="21" t="s">
+      <c r="N3" s="21" t="s">
         <v>235</v>
-      </c>
-      <c r="N3" s="21" t="s">
-        <v>236</v>
       </c>
       <c r="O3" s="21" t="s">
         <v>511</v>
       </c>
       <c r="P3" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="Q3" s="21" t="s">
         <v>237</v>
       </c>
-      <c r="Q3" s="21" t="s">
+      <c r="R3" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="R3" s="21" t="s">
+      <c r="S3" s="21" t="s">
         <v>239</v>
       </c>
-      <c r="S3" s="21" t="s">
+      <c r="T3" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="T3" s="21" t="s">
+      <c r="U3" s="21" t="s">
         <v>241</v>
       </c>
-      <c r="U3" s="21" t="s">
+      <c r="V3" s="21" t="s">
         <v>242</v>
-      </c>
-      <c r="V3" s="21" t="s">
-        <v>243</v>
       </c>
       <c r="W3" s="21" t="s">
         <v>512</v>
@@ -4768,19 +4768,19 @@
     </row>
     <row r="4" ht="34" customHeight="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" s="24" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B4" s="32" t="s">
+        <v>248</v>
+      </c>
+      <c r="C4" s="32" t="s">
+        <v>247</v>
+      </c>
+      <c r="D4" s="32" t="s">
+        <v>252</v>
+      </c>
+      <c r="E4" s="32" t="s">
         <v>249</v>
-      </c>
-      <c r="C4" s="32" t="s">
-        <v>248</v>
-      </c>
-      <c r="D4" s="32" t="s">
-        <v>253</v>
-      </c>
-      <c r="E4" s="32" t="s">
-        <v>250</v>
       </c>
       <c r="F4" s="32" t="s">
         <v>601</v>
@@ -4811,17 +4811,17 @@
       </c>
       <c r="O4" s="24"/>
       <c r="P4" s="24" t="s">
+        <v>256</v>
+      </c>
+      <c r="Q4" s="24" t="s">
         <v>257</v>
       </c>
-      <c r="Q4" s="24" t="s">
+      <c r="R4" s="24" t="s">
         <v>258</v>
-      </c>
-      <c r="R4" s="24" t="s">
-        <v>259</v>
       </c>
       <c r="S4" s="24"/>
       <c r="T4" s="24" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="U4" s="24"/>
       <c r="V4" s="24" t="s">
@@ -4839,13 +4839,13 @@
         <v>301</v>
       </c>
       <c r="C5" s="32" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D5" s="32" t="s">
         <v>304</v>
       </c>
       <c r="E5" s="32" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F5" s="32" t="s">
         <v>607</v>
@@ -4876,17 +4876,17 @@
       </c>
       <c r="O5" s="14"/>
       <c r="P5" s="14" t="s">
+        <v>256</v>
+      </c>
+      <c r="Q5" s="14" t="s">
         <v>257</v>
-      </c>
-      <c r="Q5" s="14" t="s">
-        <v>258</v>
       </c>
       <c r="R5" s="14" t="s">
         <v>308</v>
       </c>
       <c r="S5" s="14"/>
       <c r="T5" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="U5" s="14"/>
       <c r="V5" s="14" t="s">
@@ -4898,19 +4898,19 @@
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" s="24" t="s">
+        <v>272</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>274</v>
+      </c>
+      <c r="C6" s="32" t="s">
         <v>273</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="D6" s="32" t="s">
+        <v>278</v>
+      </c>
+      <c r="E6" s="32" t="s">
         <v>275</v>
-      </c>
-      <c r="C6" s="32" t="s">
-        <v>274</v>
-      </c>
-      <c r="D6" s="32" t="s">
-        <v>279</v>
-      </c>
-      <c r="E6" s="32" t="s">
-        <v>276</v>
       </c>
       <c r="F6" s="32" t="s">
         <v>415</v>
@@ -4941,17 +4941,17 @@
       </c>
       <c r="O6" s="24"/>
       <c r="P6" s="24" t="s">
+        <v>256</v>
+      </c>
+      <c r="Q6" s="24" t="s">
         <v>257</v>
       </c>
-      <c r="Q6" s="24" t="s">
-        <v>258</v>
-      </c>
       <c r="R6" s="24" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="S6" s="24"/>
       <c r="T6" s="24" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="U6" s="24"/>
       <c r="V6" s="24" t="s">
@@ -5103,7 +5103,7 @@
         <v>81</v>
       </c>
       <c r="L4" s="24" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="M4" s="24" t="s">
         <v>80</v>
@@ -5142,7 +5142,7 @@
         <v>90</v>
       </c>
       <c r="L5" s="14" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="M5" s="14"/>
     </row>
@@ -5259,7 +5259,7 @@
         <v>116</v>
       </c>
       <c r="L8" s="24" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="M8" s="24" t="s">
         <v>115</v>
@@ -5300,7 +5300,7 @@
         <v>126</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="M9" s="14" t="s">
         <v>125</v>
@@ -5571,7 +5571,7 @@
         <v>173</v>
       </c>
       <c r="L16" s="24" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="M16" s="24" t="s">
         <v>80</v>
@@ -5727,50 +5727,50 @@
         <v>186</v>
       </c>
       <c r="G6" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="H6" s="24" t="s">
         <v>198</v>
-      </c>
-      <c r="H6" s="24" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>200</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>201</v>
       </c>
       <c r="C7" s="14" t="s">
         <v>66</v>
       </c>
       <c r="D7" s="14" t="s">
+        <v>201</v>
+      </c>
+      <c r="E7" s="14" t="s">
         <v>202</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>203</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>186</v>
       </c>
       <c r="G7" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="H7" s="14" t="s">
         <v>204</v>
-      </c>
-      <c r="H7" s="14" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="24" t="s">
+        <v>205</v>
+      </c>
+      <c r="B8" s="24" t="s">
         <v>206</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="C8" s="24" t="s">
         <v>207</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="D8" s="24" t="s">
         <v>208</v>
-      </c>
-      <c r="D8" s="24" t="s">
-        <v>209</v>
       </c>
       <c r="E8" s="24" t="s">
         <v>197</v>
@@ -5779,24 +5779,24 @@
         <v>186</v>
       </c>
       <c r="G8" s="24" t="s">
+        <v>209</v>
+      </c>
+      <c r="H8" s="24" t="s">
         <v>210</v>
-      </c>
-      <c r="H8" s="24" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
+        <v>211</v>
+      </c>
+      <c r="B9" s="14" t="s">
         <v>212</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="C9" s="14" t="s">
         <v>213</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="D9" s="14" t="s">
         <v>214</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>215</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>79</v>
@@ -5805,10 +5805,10 @@
         <v>186</v>
       </c>
       <c r="G9" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="H9" s="14" t="s">
         <v>216</v>
-      </c>
-      <c r="H9" s="14" t="s">
-        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -5878,7 +5878,7 @@
         <v>631</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C5" s="14" t="s">
         <v>632</v>
@@ -5886,7 +5886,7 @@
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="24" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B6" s="24">
         <v>6</v>
@@ -5897,7 +5897,7 @@
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B7" s="14">
         <v>2</v>
@@ -6050,7 +6050,7 @@
         <v>659</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C4" s="24" t="s">
         <v>660</v>
@@ -6202,7 +6202,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -6231,7 +6231,7 @@
     </row>
     <row r="2" ht="34" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B2" s="20"/>
       <c r="C2" s="20"/>
@@ -6263,120 +6263,120 @@
         <v>175</v>
       </c>
       <c r="B3" s="21" t="s">
+        <v>219</v>
+      </c>
+      <c r="C3" s="21" t="s">
         <v>220</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="D3" s="21" t="s">
         <v>221</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="E3" s="21" t="s">
         <v>222</v>
       </c>
-      <c r="E3" s="21" t="s">
+      <c r="F3" s="21" t="s">
         <v>223</v>
       </c>
-      <c r="F3" s="21" t="s">
+      <c r="G3" s="21" t="s">
         <v>224</v>
       </c>
-      <c r="G3" s="21" t="s">
+      <c r="H3" s="21" t="s">
         <v>225</v>
       </c>
-      <c r="H3" s="21" t="s">
+      <c r="I3" s="21" t="s">
         <v>226</v>
       </c>
-      <c r="I3" s="21" t="s">
+      <c r="J3" s="21" t="s">
         <v>227</v>
       </c>
-      <c r="J3" s="21" t="s">
+      <c r="K3" s="21" t="s">
         <v>228</v>
       </c>
-      <c r="K3" s="21" t="s">
+      <c r="L3" s="21" t="s">
         <v>229</v>
       </c>
-      <c r="L3" s="21" t="s">
+      <c r="M3" s="22" t="s">
         <v>230</v>
       </c>
-      <c r="M3" s="22" t="s">
+      <c r="N3" s="21" t="s">
         <v>231</v>
       </c>
-      <c r="N3" s="21" t="s">
+      <c r="O3" s="23" t="s">
         <v>232</v>
       </c>
-      <c r="O3" s="23" t="s">
+      <c r="P3" s="21" t="s">
         <v>233</v>
       </c>
-      <c r="P3" s="21" t="s">
+      <c r="Q3" s="21" t="s">
         <v>234</v>
       </c>
-      <c r="Q3" s="21" t="s">
+      <c r="R3" s="21" t="s">
         <v>235</v>
       </c>
-      <c r="R3" s="21" t="s">
+      <c r="S3" s="21" t="s">
         <v>236</v>
       </c>
-      <c r="S3" s="21" t="s">
+      <c r="T3" s="21" t="s">
         <v>237</v>
       </c>
-      <c r="T3" s="21" t="s">
+      <c r="U3" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="U3" s="21" t="s">
+      <c r="V3" s="21" t="s">
         <v>239</v>
       </c>
-      <c r="V3" s="21" t="s">
+      <c r="W3" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="W3" s="21" t="s">
+      <c r="X3" s="21" t="s">
         <v>241</v>
       </c>
-      <c r="X3" s="21" t="s">
+      <c r="Y3" s="21" t="s">
         <v>242</v>
-      </c>
-      <c r="Y3" s="21" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="4" ht="34" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" s="24" t="s">
+        <v>243</v>
+      </c>
+      <c r="B4" s="24" t="s">
         <v>244</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="C4" s="25" t="s">
         <v>245</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="D4" s="24" t="s">
         <v>246</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="E4" s="24" t="s">
         <v>247</v>
       </c>
-      <c r="E4" s="24" t="s">
+      <c r="F4" s="24" t="s">
         <v>248</v>
       </c>
-      <c r="F4" s="24" t="s">
+      <c r="G4" s="24" t="s">
         <v>249</v>
       </c>
-      <c r="G4" s="24" t="s">
+      <c r="H4" s="24" t="s">
         <v>250</v>
       </c>
-      <c r="H4" s="24" t="s">
+      <c r="I4" s="24" t="s">
         <v>251</v>
       </c>
-      <c r="I4" s="24" t="s">
+      <c r="J4" s="24" t="s">
         <v>252</v>
       </c>
-      <c r="J4" s="24" t="s">
+      <c r="K4" s="24" t="s">
         <v>253</v>
       </c>
-      <c r="K4" s="24" t="s">
+      <c r="L4" s="24" t="s">
         <v>254</v>
-      </c>
-      <c r="L4" s="24" t="s">
-        <v>255</v>
       </c>
       <c r="M4" s="26">
         <v>1</v>
       </c>
       <c r="N4" s="24" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="O4" s="27">
         <v>5</v>
@@ -6391,17 +6391,17 @@
         <v>0</v>
       </c>
       <c r="S4" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="T4" s="25" t="s">
         <v>257</v>
       </c>
-      <c r="T4" s="25" t="s">
+      <c r="U4" s="28" t="s">
         <v>258</v>
-      </c>
-      <c r="U4" s="28" t="s">
-        <v>259</v>
       </c>
       <c r="V4" s="24"/>
       <c r="W4" s="24" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="X4" s="24"/>
       <c r="Y4" s="24" t="s">
@@ -6410,46 +6410,46 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="B5" s="14" t="s">
         <v>261</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="C5" s="25" t="s">
+        <v>245</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="E5" s="14" t="s">
         <v>262</v>
       </c>
-      <c r="C5" s="25" t="s">
-        <v>246</v>
-      </c>
-      <c r="D5" s="14" t="s">
-        <v>214</v>
-      </c>
-      <c r="E5" s="14" t="s">
+      <c r="F5" s="14" t="s">
         <v>263</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="G5" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="H5" s="14" t="s">
         <v>265</v>
       </c>
-      <c r="H5" s="14" t="s">
+      <c r="I5" s="14" t="s">
         <v>266</v>
       </c>
-      <c r="I5" s="14" t="s">
+      <c r="J5" s="14" t="s">
         <v>267</v>
       </c>
-      <c r="J5" s="14" t="s">
+      <c r="K5" s="14" t="s">
         <v>268</v>
       </c>
-      <c r="K5" s="14" t="s">
+      <c r="L5" s="14" t="s">
         <v>269</v>
-      </c>
-      <c r="L5" s="14" t="s">
-        <v>270</v>
       </c>
       <c r="M5" s="26">
         <v>1</v>
       </c>
       <c r="N5" s="14" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="O5" s="29">
         <v>4.9</v>
@@ -6464,17 +6464,17 @@
         <v>0</v>
       </c>
       <c r="S5" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="T5" s="25" t="s">
         <v>257</v>
       </c>
-      <c r="T5" s="25" t="s">
-        <v>258</v>
-      </c>
       <c r="U5" s="28" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="V5" s="14"/>
       <c r="W5" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="X5" s="14"/>
       <c r="Y5" s="14" t="s">
@@ -6483,46 +6483,46 @@
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" s="24" t="s">
+        <v>272</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>244</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>245</v>
+      </c>
+      <c r="D6" s="24" t="s">
+        <v>246</v>
+      </c>
+      <c r="E6" s="24" t="s">
         <v>273</v>
       </c>
-      <c r="B6" s="24" t="s">
-        <v>245</v>
-      </c>
-      <c r="C6" s="25" t="s">
-        <v>246</v>
-      </c>
-      <c r="D6" s="24" t="s">
-        <v>247</v>
-      </c>
-      <c r="E6" s="24" t="s">
+      <c r="F6" s="24" t="s">
         <v>274</v>
       </c>
-      <c r="F6" s="24" t="s">
+      <c r="G6" s="24" t="s">
         <v>275</v>
       </c>
-      <c r="G6" s="24" t="s">
+      <c r="H6" s="24" t="s">
         <v>276</v>
       </c>
-      <c r="H6" s="24" t="s">
+      <c r="I6" s="24" t="s">
         <v>277</v>
       </c>
-      <c r="I6" s="24" t="s">
+      <c r="J6" s="24" t="s">
         <v>278</v>
       </c>
-      <c r="J6" s="24" t="s">
+      <c r="K6" s="24" t="s">
         <v>279</v>
       </c>
-      <c r="K6" s="24" t="s">
+      <c r="L6" s="24" t="s">
         <v>280</v>
-      </c>
-      <c r="L6" s="24" t="s">
-        <v>281</v>
       </c>
       <c r="M6" s="26">
         <v>1</v>
       </c>
       <c r="N6" s="24" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="O6" s="27">
         <v>4.8</v>
@@ -6537,17 +6537,17 @@
         <v>0</v>
       </c>
       <c r="S6" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="T6" s="25" t="s">
         <v>257</v>
       </c>
-      <c r="T6" s="25" t="s">
-        <v>258</v>
-      </c>
       <c r="U6" s="28" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="V6" s="24"/>
       <c r="W6" s="24" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="X6" s="24"/>
       <c r="Y6" s="24" t="s">
@@ -6556,46 +6556,46 @@
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
+        <v>283</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>284</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="C7" s="25" t="s">
         <v>285</v>
-      </c>
-      <c r="C7" s="25" t="s">
-        <v>286</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>84</v>
       </c>
       <c r="E7" s="14" t="s">
+        <v>286</v>
+      </c>
+      <c r="F7" s="14" t="s">
         <v>287</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="G7" s="14" t="s">
         <v>288</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="H7" s="14" t="s">
         <v>289</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="I7" s="14" t="s">
         <v>290</v>
       </c>
-      <c r="I7" s="14" t="s">
+      <c r="J7" s="14" t="s">
         <v>291</v>
       </c>
-      <c r="J7" s="14" t="s">
+      <c r="K7" s="14" t="s">
         <v>292</v>
       </c>
-      <c r="K7" s="14" t="s">
+      <c r="L7" s="14" t="s">
         <v>293</v>
-      </c>
-      <c r="L7" s="14" t="s">
-        <v>294</v>
       </c>
       <c r="M7" s="26">
         <v>1</v>
       </c>
       <c r="N7" s="14" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="O7" s="29">
         <v>4.8</v>
@@ -6610,15 +6610,17 @@
         <v>0</v>
       </c>
       <c r="S7" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="T7" s="25" t="s">
         <v>257</v>
       </c>
-      <c r="T7" s="25" t="s">
-        <v>258</v>
-      </c>
       <c r="U7" s="28" t="s">
+        <v>295</v>
+      </c>
+      <c r="V7" s="14" t="s">
         <v>296</v>
       </c>
-      <c r="V7" s="14"/>
       <c r="W7" s="14" t="s">
         <v>297</v>
       </c>
@@ -6632,22 +6634,22 @@
         <v>299</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C8" s="25" t="s">
         <v>300</v>
       </c>
       <c r="D8" s="24" t="s">
+        <v>246</v>
+      </c>
+      <c r="E8" s="24" t="s">
         <v>247</v>
-      </c>
-      <c r="E8" s="24" t="s">
-        <v>248</v>
       </c>
       <c r="F8" s="24" t="s">
         <v>301</v>
       </c>
       <c r="G8" s="24" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="H8" s="24" t="s">
         <v>302</v>
@@ -6683,17 +6685,17 @@
         <v>0</v>
       </c>
       <c r="S8" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="T8" s="25" t="s">
         <v>257</v>
-      </c>
-      <c r="T8" s="25" t="s">
-        <v>258</v>
       </c>
       <c r="U8" s="28" t="s">
         <v>308</v>
       </c>
       <c r="V8" s="24"/>
       <c r="W8" s="24" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="X8" s="24"/>
       <c r="Y8" s="24" t="s">
@@ -6705,13 +6707,13 @@
         <v>310</v>
       </c>
       <c r="B9" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="C9" s="25" t="s">
         <v>285</v>
       </c>
-      <c r="C9" s="25" t="s">
-        <v>286</v>
-      </c>
       <c r="D9" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>311</v>
@@ -6756,10 +6758,10 @@
         <v>0</v>
       </c>
       <c r="S9" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="T9" s="25" t="s">
         <v>257</v>
-      </c>
-      <c r="T9" s="25" t="s">
-        <v>258</v>
       </c>
       <c r="U9" s="28" t="s">
         <v>320</v>
@@ -6778,22 +6780,22 @@
         <v>322</v>
       </c>
       <c r="B10" s="24" t="s">
+        <v>261</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>245</v>
+      </c>
+      <c r="D10" s="24" t="s">
+        <v>213</v>
+      </c>
+      <c r="E10" s="24" t="s">
         <v>262</v>
-      </c>
-      <c r="C10" s="25" t="s">
-        <v>246</v>
-      </c>
-      <c r="D10" s="24" t="s">
-        <v>214</v>
-      </c>
-      <c r="E10" s="24" t="s">
-        <v>263</v>
       </c>
       <c r="F10" s="24" t="s">
         <v>323</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="H10" s="24" t="s">
         <v>324</v>
@@ -6829,17 +6831,17 @@
         <v>0</v>
       </c>
       <c r="S10" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="T10" s="25" t="s">
         <v>257</v>
-      </c>
-      <c r="T10" s="25" t="s">
-        <v>258</v>
       </c>
       <c r="U10" s="28" t="s">
         <v>330</v>
       </c>
       <c r="V10" s="24"/>
       <c r="W10" s="24" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="X10" s="24"/>
       <c r="Y10" s="24" t="s">
@@ -6851,16 +6853,16 @@
         <v>331</v>
       </c>
       <c r="B11" s="14" t="s">
+        <v>261</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>245</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="E11" s="14" t="s">
         <v>262</v>
-      </c>
-      <c r="C11" s="25" t="s">
-        <v>246</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>214</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>263</v>
       </c>
       <c r="F11" s="14" t="s">
         <v>332</v>
@@ -6902,17 +6904,17 @@
         <v>0</v>
       </c>
       <c r="S11" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="T11" s="25" t="s">
         <v>257</v>
-      </c>
-      <c r="T11" s="25" t="s">
-        <v>258</v>
       </c>
       <c r="U11" s="28" t="s">
         <v>340</v>
       </c>
       <c r="V11" s="14"/>
       <c r="W11" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="X11" s="14"/>
       <c r="Y11" s="14" t="s">
@@ -6924,13 +6926,13 @@
         <v>341</v>
       </c>
       <c r="B12" s="24" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D12" s="24" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E12" s="24" t="s">
         <v>342</v>
@@ -6939,7 +6941,7 @@
         <v>343</v>
       </c>
       <c r="G12" s="24" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="H12" s="24" t="s">
         <v>344</v>
@@ -6975,17 +6977,17 @@
         <v>0</v>
       </c>
       <c r="S12" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="T12" s="25" t="s">
         <v>257</v>
-      </c>
-      <c r="T12" s="25" t="s">
-        <v>258</v>
       </c>
       <c r="U12" s="28" t="s">
         <v>350</v>
       </c>
       <c r="V12" s="24"/>
       <c r="W12" s="24" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="X12" s="24"/>
       <c r="Y12" s="24" t="s">
@@ -6997,13 +6999,13 @@
         <v>351</v>
       </c>
       <c r="B13" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="C13" s="25" t="s">
         <v>285</v>
       </c>
-      <c r="C13" s="25" t="s">
-        <v>286</v>
-      </c>
       <c r="D13" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E13" s="14" t="s">
         <v>352</v>
@@ -7048,10 +7050,10 @@
         <v>0</v>
       </c>
       <c r="S13" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="T13" s="25" t="s">
         <v>257</v>
-      </c>
-      <c r="T13" s="25" t="s">
-        <v>258</v>
       </c>
       <c r="U13" s="28" t="s">
         <v>359</v>
@@ -7070,16 +7072,16 @@
         <v>360</v>
       </c>
       <c r="B14" s="24" t="s">
+        <v>284</v>
+      </c>
+      <c r="C14" s="25" t="s">
         <v>285</v>
       </c>
-      <c r="C14" s="25" t="s">
-        <v>286</v>
-      </c>
       <c r="D14" s="24" t="s">
+        <v>246</v>
+      </c>
+      <c r="E14" s="24" t="s">
         <v>247</v>
-      </c>
-      <c r="E14" s="24" t="s">
-        <v>248</v>
       </c>
       <c r="F14" s="24" t="s">
         <v>361</v>
@@ -7244,7 +7246,7 @@
         <v>175</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C3" s="21" t="s">
         <v>374</v>
@@ -7259,13 +7261,13 @@
         <v>377</v>
       </c>
       <c r="G3" s="21" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H3" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="I3" s="21" t="s">
         <v>222</v>
-      </c>
-      <c r="I3" s="21" t="s">
-        <v>223</v>
       </c>
       <c r="J3" s="21" t="s">
         <v>378</v>
@@ -7283,7 +7285,7 @@
         <v>382</v>
       </c>
       <c r="O3" s="21" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="P3" s="21" t="s">
         <v>383</v>
@@ -7319,10 +7321,10 @@
       </c>
       <c r="G4" s="24"/>
       <c r="H4" s="24" t="s">
+        <v>246</v>
+      </c>
+      <c r="I4" s="24" t="s">
         <v>247</v>
-      </c>
-      <c r="I4" s="24" t="s">
-        <v>248</v>
       </c>
       <c r="J4" s="24" t="s">
         <v>390</v>
@@ -7356,7 +7358,7 @@
         <v>396</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C5" s="14" t="s">
         <v>397</v>
@@ -7374,10 +7376,10 @@
         <v>80</v>
       </c>
       <c r="H5" s="14" t="s">
+        <v>246</v>
+      </c>
+      <c r="I5" s="14" t="s">
         <v>247</v>
-      </c>
-      <c r="I5" s="14" t="s">
-        <v>248</v>
       </c>
       <c r="J5" s="14" t="s">
         <v>400</v>
@@ -7395,7 +7397,7 @@
         <v>401</v>
       </c>
       <c r="O5" s="14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="P5" s="14" t="s">
         <v>402</v>
@@ -7413,7 +7415,7 @@
         <v>405</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C6" s="24" t="s">
         <v>406</v>
@@ -7431,10 +7433,10 @@
         <v>309</v>
       </c>
       <c r="H6" s="24" t="s">
+        <v>246</v>
+      </c>
+      <c r="I6" s="24" t="s">
         <v>247</v>
-      </c>
-      <c r="I6" s="24" t="s">
-        <v>248</v>
       </c>
       <c r="J6" s="24" t="s">
         <v>400</v>
@@ -7470,7 +7472,7 @@
         <v>411</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C7" s="14" t="s">
         <v>412</v>
@@ -7488,10 +7490,10 @@
         <v>115</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I7" s="14" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="J7" s="14" t="s">
         <v>400</v>
@@ -7509,7 +7511,7 @@
         <v>414</v>
       </c>
       <c r="O7" s="14" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="P7" s="14" t="s">
         <v>415</v>
@@ -7527,7 +7529,7 @@
         <v>417</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>418</v>
@@ -7545,10 +7547,10 @@
         <v>125</v>
       </c>
       <c r="H8" s="24" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="I8" s="24" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="J8" s="24" t="s">
         <v>400</v>
@@ -7566,7 +7568,7 @@
         <v>420</v>
       </c>
       <c r="O8" s="24" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="P8" s="24" t="s">
         <v>421</v>
@@ -7584,7 +7586,7 @@
         <v>423</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C9" s="14" t="s">
         <v>424</v>
@@ -7602,10 +7604,10 @@
         <v>140</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="J9" s="14" t="s">
         <v>400</v>
@@ -7641,7 +7643,7 @@
         <v>429</v>
       </c>
       <c r="B10" s="24" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C10" s="24" t="s">
         <v>430</v>
@@ -7659,7 +7661,7 @@
         <v>99</v>
       </c>
       <c r="H10" s="24" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="I10" s="24" t="s">
         <v>342</v>
@@ -7698,7 +7700,7 @@
         <v>435</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C11" s="14" t="s">
         <v>436</v>
@@ -7716,10 +7718,10 @@
         <v>162</v>
       </c>
       <c r="H11" s="14" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="I11" s="14" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="J11" s="14" t="s">
         <v>400</v>
@@ -7767,14 +7769,14 @@
         <v>298</v>
       </c>
       <c r="F12" s="24" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="G12" s="24"/>
       <c r="H12" s="24" t="s">
         <v>84</v>
       </c>
       <c r="I12" s="24" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J12" s="24" t="s">
         <v>390</v>
@@ -7792,7 +7794,7 @@
         <v>444</v>
       </c>
       <c r="O12" s="24" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="P12" s="24" t="s">
         <v>445</v>
@@ -7826,7 +7828,7 @@
       </c>
       <c r="G13" s="14"/>
       <c r="H13" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="I13" s="14" t="s">
         <v>352</v>
@@ -7941,7 +7943,7 @@
         <v>175</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C3" s="21" t="s">
         <v>375</v>
@@ -7953,10 +7955,10 @@
         <v>376</v>
       </c>
       <c r="F3" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="G3" s="21" t="s">
         <v>222</v>
-      </c>
-      <c r="G3" s="21" t="s">
-        <v>223</v>
       </c>
       <c r="H3" s="21" t="s">
         <v>378</v>
@@ -7974,13 +7976,13 @@
         <v>382</v>
       </c>
       <c r="M3" s="21" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="N3" s="21" t="s">
         <v>385</v>
       </c>
       <c r="O3" s="21" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="P3" s="21" t="s">
         <v>458</v>
@@ -8003,10 +8005,10 @@
         <v>371</v>
       </c>
       <c r="F4" s="24" t="s">
+        <v>246</v>
+      </c>
+      <c r="G4" s="24" t="s">
         <v>247</v>
-      </c>
-      <c r="G4" s="24" t="s">
-        <v>248</v>
       </c>
       <c r="H4" s="24" t="s">
         <v>390</v>
@@ -8037,7 +8039,7 @@
         <v>396</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C5" s="14" t="s">
         <v>398</v>
@@ -8047,10 +8049,10 @@
       </c>
       <c r="E5" s="14"/>
       <c r="F5" s="14" t="s">
+        <v>246</v>
+      </c>
+      <c r="G5" s="14" t="s">
         <v>247</v>
-      </c>
-      <c r="G5" s="14" t="s">
-        <v>248</v>
       </c>
       <c r="H5" s="14" t="s">
         <v>400</v>
@@ -8068,7 +8070,7 @@
         <v>401</v>
       </c>
       <c r="M5" s="14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="N5" s="14"/>
       <c r="O5" s="14" t="s">
@@ -8083,7 +8085,7 @@
         <v>405</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C6" s="24" t="s">
         <v>398</v>
@@ -8093,10 +8095,10 @@
       </c>
       <c r="E6" s="24"/>
       <c r="F6" s="24" t="s">
+        <v>246</v>
+      </c>
+      <c r="G6" s="24" t="s">
         <v>247</v>
-      </c>
-      <c r="G6" s="24" t="s">
-        <v>248</v>
       </c>
       <c r="H6" s="24" t="s">
         <v>400</v>
@@ -8129,7 +8131,7 @@
         <v>411</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C7" s="14" t="s">
         <v>398</v>
@@ -8139,10 +8141,10 @@
       </c>
       <c r="E7" s="14"/>
       <c r="F7" s="14" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="H7" s="14" t="s">
         <v>400</v>
@@ -8160,7 +8162,7 @@
         <v>414</v>
       </c>
       <c r="M7" s="14" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="N7" s="14"/>
       <c r="O7" s="14" t="s">
@@ -8175,7 +8177,7 @@
         <v>417</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>398</v>
@@ -8185,10 +8187,10 @@
       </c>
       <c r="E8" s="24"/>
       <c r="F8" s="24" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G8" s="24" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="H8" s="24" t="s">
         <v>400</v>
@@ -8206,7 +8208,7 @@
         <v>420</v>
       </c>
       <c r="M8" s="24" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="N8" s="24"/>
       <c r="O8" s="24" t="s">
@@ -8221,7 +8223,7 @@
         <v>423</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C9" s="14" t="s">
         <v>398</v>
@@ -8231,10 +8233,10 @@
       </c>
       <c r="E9" s="14"/>
       <c r="F9" s="14" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="H9" s="14" t="s">
         <v>400</v>
@@ -8267,7 +8269,7 @@
         <v>429</v>
       </c>
       <c r="B10" s="24" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C10" s="24" t="s">
         <v>398</v>
@@ -8277,7 +8279,7 @@
       </c>
       <c r="E10" s="24"/>
       <c r="F10" s="24" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G10" s="24" t="s">
         <v>342</v>
@@ -8313,7 +8315,7 @@
         <v>435</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C11" s="14" t="s">
         <v>398</v>
@@ -8323,10 +8325,10 @@
       </c>
       <c r="E11" s="14"/>
       <c r="F11" s="14" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="H11" s="14" t="s">
         <v>400</v>
@@ -8365,7 +8367,7 @@
         <v>443</v>
       </c>
       <c r="D12" s="24" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E12" s="24" t="s">
         <v>298</v>
@@ -8374,7 +8376,7 @@
         <v>84</v>
       </c>
       <c r="G12" s="24" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="H12" s="24" t="s">
         <v>390</v>
@@ -8392,7 +8394,7 @@
         <v>444</v>
       </c>
       <c r="M12" s="24" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="N12" s="24"/>
       <c r="O12" s="24"/>
@@ -8417,7 +8419,7 @@
         <v>321</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G13" s="14" t="s">
         <v>352</v>
@@ -8485,7 +8487,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="30" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B1" s="30"/>
       <c r="C1" s="30"/>
@@ -8533,10 +8535,10 @@
         <v>463</v>
       </c>
       <c r="C3" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="D3" s="21" t="s">
         <v>222</v>
-      </c>
-      <c r="D3" s="21" t="s">
-        <v>223</v>
       </c>
       <c r="E3" s="21" t="s">
         <v>464</v>
@@ -8563,19 +8565,19 @@
         <v>375</v>
       </c>
       <c r="M3" s="21" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="N3" s="21" t="s">
         <v>380</v>
       </c>
       <c r="O3" s="21" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="P3" s="21" t="s">
         <v>471</v>
       </c>
       <c r="Q3" s="21" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" ht="34" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
@@ -8586,10 +8588,10 @@
         <v>361</v>
       </c>
       <c r="C4" s="32" t="s">
+        <v>246</v>
+      </c>
+      <c r="D4" s="32" t="s">
         <v>247</v>
-      </c>
-      <c r="D4" s="32" t="s">
-        <v>248</v>
       </c>
       <c r="E4" s="32" t="s">
         <v>365</v>
@@ -8631,25 +8633,25 @@
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B5" s="32" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C5" s="32" t="s">
         <v>84</v>
       </c>
       <c r="D5" s="32" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E5" s="32" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F5" s="32" t="s">
+        <v>288</v>
+      </c>
+      <c r="G5" s="32" t="s">
         <v>289</v>
-      </c>
-      <c r="G5" s="32" t="s">
-        <v>290</v>
       </c>
       <c r="H5" s="32" t="s">
         <v>474</v>
@@ -8673,13 +8675,13 @@
         <v>461</v>
       </c>
       <c r="O5" s="14" t="s">
+        <v>256</v>
+      </c>
+      <c r="P5" s="14" t="s">
         <v>257</v>
       </c>
-      <c r="P5" s="14" t="s">
-        <v>258</v>
-      </c>
       <c r="Q5" s="14" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
@@ -8690,7 +8692,7 @@
         <v>312</v>
       </c>
       <c r="C6" s="32" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D6" s="32" t="s">
         <v>311</v>
@@ -8726,10 +8728,10 @@
         <v>461</v>
       </c>
       <c r="O6" s="24" t="s">
+        <v>256</v>
+      </c>
+      <c r="P6" s="24" t="s">
         <v>257</v>
-      </c>
-      <c r="P6" s="24" t="s">
-        <v>258</v>
       </c>
       <c r="Q6" s="24" t="s">
         <v>320</v>
@@ -8743,7 +8745,7 @@
         <v>353</v>
       </c>
       <c r="C7" s="32" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D7" s="32" t="s">
         <v>352</v>
@@ -8779,10 +8781,10 @@
         <v>461</v>
       </c>
       <c r="O7" s="14" t="s">
+        <v>256</v>
+      </c>
+      <c r="P7" s="14" t="s">
         <v>257</v>
-      </c>
-      <c r="P7" s="14" t="s">
-        <v>258</v>
       </c>
       <c r="Q7" s="14" t="s">
         <v>359</v>
@@ -8961,13 +8963,13 @@
         <v>175</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E3" s="21" t="s">
         <v>487</v>
@@ -9060,46 +9062,46 @@
         <v>509</v>
       </c>
       <c r="AI3" s="22" t="s">
+        <v>230</v>
+      </c>
+      <c r="AJ3" s="21" t="s">
         <v>231</v>
-      </c>
-      <c r="AJ3" s="21" t="s">
-        <v>232</v>
       </c>
       <c r="AK3" s="21" t="s">
         <v>510</v>
       </c>
       <c r="AL3" s="21" t="s">
+        <v>233</v>
+      </c>
+      <c r="AM3" s="21" t="s">
         <v>234</v>
       </c>
-      <c r="AM3" s="21" t="s">
+      <c r="AN3" s="21" t="s">
         <v>235</v>
-      </c>
-      <c r="AN3" s="21" t="s">
-        <v>236</v>
       </c>
       <c r="AO3" s="21" t="s">
         <v>511</v>
       </c>
       <c r="AP3" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="AQ3" s="21" t="s">
         <v>237</v>
       </c>
-      <c r="AQ3" s="21" t="s">
+      <c r="AR3" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="AR3" s="21" t="s">
+      <c r="AS3" s="21" t="s">
         <v>239</v>
       </c>
-      <c r="AS3" s="21" t="s">
+      <c r="AT3" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="AT3" s="21" t="s">
+      <c r="AU3" s="21" t="s">
         <v>241</v>
       </c>
-      <c r="AU3" s="21" t="s">
+      <c r="AV3" s="21" t="s">
         <v>242</v>
-      </c>
-      <c r="AV3" s="21" t="s">
-        <v>243</v>
       </c>
       <c r="AW3" s="21" t="s">
         <v>512</v>
@@ -9241,13 +9243,13 @@
         <v>175</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E3" s="21" t="s">
         <v>515</v>
@@ -9304,46 +9306,46 @@
         <v>509</v>
       </c>
       <c r="W3" s="22" t="s">
+        <v>230</v>
+      </c>
+      <c r="X3" s="21" t="s">
         <v>231</v>
-      </c>
-      <c r="X3" s="21" t="s">
-        <v>232</v>
       </c>
       <c r="Y3" s="21" t="s">
         <v>510</v>
       </c>
       <c r="Z3" s="21" t="s">
+        <v>233</v>
+      </c>
+      <c r="AA3" s="21" t="s">
         <v>234</v>
       </c>
-      <c r="AA3" s="21" t="s">
+      <c r="AB3" s="21" t="s">
         <v>235</v>
-      </c>
-      <c r="AB3" s="21" t="s">
-        <v>236</v>
       </c>
       <c r="AC3" s="21" t="s">
         <v>511</v>
       </c>
       <c r="AD3" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="AE3" s="21" t="s">
         <v>237</v>
       </c>
-      <c r="AE3" s="21" t="s">
+      <c r="AF3" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="AF3" s="21" t="s">
+      <c r="AG3" s="21" t="s">
         <v>239</v>
       </c>
-      <c r="AG3" s="21" t="s">
+      <c r="AH3" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="AH3" s="21" t="s">
+      <c r="AI3" s="21" t="s">
         <v>241</v>
       </c>
-      <c r="AI3" s="21" t="s">
+      <c r="AJ3" s="21" t="s">
         <v>242</v>
-      </c>
-      <c r="AJ3" s="21" t="s">
-        <v>243</v>
       </c>
       <c r="AK3" s="21" t="s">
         <v>512</v>
@@ -9503,16 +9505,16 @@
         <v>175</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C3" s="21" t="s">
         <v>526</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E3" s="21" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F3" s="21" t="s">
         <v>487</v>
@@ -9590,46 +9592,46 @@
         <v>509</v>
       </c>
       <c r="AE3" s="22" t="s">
+        <v>230</v>
+      </c>
+      <c r="AF3" s="21" t="s">
         <v>231</v>
-      </c>
-      <c r="AF3" s="21" t="s">
-        <v>232</v>
       </c>
       <c r="AG3" s="21" t="s">
         <v>510</v>
       </c>
       <c r="AH3" s="21" t="s">
+        <v>233</v>
+      </c>
+      <c r="AI3" s="21" t="s">
         <v>234</v>
       </c>
-      <c r="AI3" s="21" t="s">
+      <c r="AJ3" s="21" t="s">
         <v>235</v>
-      </c>
-      <c r="AJ3" s="21" t="s">
-        <v>236</v>
       </c>
       <c r="AK3" s="21" t="s">
         <v>511</v>
       </c>
       <c r="AL3" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="AM3" s="21" t="s">
         <v>237</v>
       </c>
-      <c r="AM3" s="21" t="s">
+      <c r="AN3" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="AN3" s="21" t="s">
+      <c r="AO3" s="21" t="s">
         <v>239</v>
       </c>
-      <c r="AO3" s="21" t="s">
+      <c r="AP3" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="AP3" s="21" t="s">
+      <c r="AQ3" s="21" t="s">
         <v>241</v>
       </c>
-      <c r="AQ3" s="21" t="s">
+      <c r="AR3" s="21" t="s">
         <v>242</v>
-      </c>
-      <c r="AR3" s="21" t="s">
-        <v>243</v>
       </c>
       <c r="AS3" s="21" t="s">
         <v>512</v>
@@ -9782,13 +9784,13 @@
         <v>175</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E3" s="21" t="s">
         <v>487</v>
@@ -9857,46 +9859,46 @@
         <v>509</v>
       </c>
       <c r="AA3" s="22" t="s">
+        <v>230</v>
+      </c>
+      <c r="AB3" s="21" t="s">
         <v>231</v>
-      </c>
-      <c r="AB3" s="21" t="s">
-        <v>232</v>
       </c>
       <c r="AC3" s="21" t="s">
         <v>510</v>
       </c>
       <c r="AD3" s="21" t="s">
+        <v>233</v>
+      </c>
+      <c r="AE3" s="21" t="s">
         <v>234</v>
       </c>
-      <c r="AE3" s="21" t="s">
+      <c r="AF3" s="21" t="s">
         <v>235</v>
-      </c>
-      <c r="AF3" s="21" t="s">
-        <v>236</v>
       </c>
       <c r="AG3" s="21" t="s">
         <v>511</v>
       </c>
       <c r="AH3" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="AI3" s="21" t="s">
         <v>237</v>
       </c>
-      <c r="AI3" s="21" t="s">
+      <c r="AJ3" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="AJ3" s="21" t="s">
+      <c r="AK3" s="21" t="s">
         <v>239</v>
       </c>
-      <c r="AK3" s="21" t="s">
+      <c r="AL3" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="AL3" s="21" t="s">
+      <c r="AM3" s="21" t="s">
         <v>241</v>
       </c>
-      <c r="AM3" s="21" t="s">
+      <c r="AN3" s="21" t="s">
         <v>242</v>
-      </c>
-      <c r="AN3" s="21" t="s">
-        <v>243</v>
       </c>
       <c r="AO3" s="21" t="s">
         <v>512</v>

</xml_diff>